<commit_message>
Reassign fleet_management@mccoys.com work orders to John Grimsley
4 work orders previously under the shared fleet_management@mccoys.com
account are reassigned to John Grimsley per standing instruction.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CrwetQk1auhq4UUVQCe1Ph
</commit_message>
<xml_diff>
--- a/Fleet_Team_WO_Follow_Up_10_13_2026_cleaned.xlsx
+++ b/Fleet_Team_WO_Follow_Up_10_13_2026_cleaned.xlsx
@@ -40314,7 +40314,7 @@
       </c>
       <c r="C524" t="inlineStr">
         <is>
-          <t>fleet_management@mccoys.com</t>
+          <t>John Grimsley</t>
         </is>
       </c>
       <c r="D524" t="inlineStr">
@@ -41222,7 +41222,7 @@
       </c>
       <c r="C539" t="inlineStr">
         <is>
-          <t>fleet_management@mccoys.com</t>
+          <t>John Grimsley</t>
         </is>
       </c>
       <c r="D539" t="inlineStr">
@@ -41283,7 +41283,7 @@
       </c>
       <c r="C540" t="inlineStr">
         <is>
-          <t>fleet_management@mccoys.com</t>
+          <t>John Grimsley</t>
         </is>
       </c>
       <c r="D540" t="inlineStr">
@@ -41344,7 +41344,7 @@
       </c>
       <c r="C541" t="inlineStr">
         <is>
-          <t>fleet_management@mccoys.com</t>
+          <t>John Grimsley</t>
         </is>
       </c>
       <c r="D541" t="inlineStr">

</xml_diff>